<commit_message>
Day 35: Add portfolio summary PDF report
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Cash Flow Intelligence" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="cashflow_intelligence" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,11 @@
           <t>capital_allocation_label</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>capital_allocation_pattern</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -513,6 +518,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -554,6 +564,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -595,6 +610,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -636,6 +656,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -677,6 +702,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -718,6 +748,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -731,17 +766,9 @@
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="b">
@@ -755,6 +782,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -796,6 +828,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -837,6 +874,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -876,6 +918,11 @@
       <c r="K11" t="inlineStr">
         <is>
           <t>Balanced</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -919,6 +966,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -958,6 +1010,11 @@
       <c r="K13" t="inlineStr">
         <is>
           <t>Asset Light</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1001,6 +1058,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1040,6 +1102,11 @@
       <c r="K15" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1083,6 +1150,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1124,6 +1196,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1165,6 +1242,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1204,6 +1286,11 @@
       <c r="K19" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1247,6 +1334,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Distress Signal</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1288,6 +1380,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1329,6 +1426,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1370,6 +1472,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1409,6 +1516,11 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>Asset Light</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -1452,6 +1564,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1493,6 +1610,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1534,6 +1656,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1575,6 +1702,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1616,6 +1748,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1657,6 +1794,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1698,6 +1840,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1739,6 +1886,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1780,6 +1932,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1821,6 +1978,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1860,6 +2022,11 @@
       <c r="K35" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Mixed</t>
         </is>
       </c>
     </row>
@@ -1903,6 +2070,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1944,6 +2116,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1985,6 +2162,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2026,6 +2208,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2067,6 +2254,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2108,6 +2300,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2149,6 +2346,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2190,6 +2392,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2231,6 +2438,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2272,6 +2484,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2313,6 +2530,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2354,6 +2576,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2395,6 +2622,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2436,6 +2668,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Pre-Revenue</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2477,6 +2714,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2518,6 +2760,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2559,6 +2806,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2600,6 +2852,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2641,6 +2898,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2682,6 +2944,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2723,6 +2990,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2764,6 +3036,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2805,6 +3082,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2846,6 +3128,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2887,6 +3174,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2928,6 +3220,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2969,6 +3266,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3008,6 +3310,11 @@
       <c r="K63" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3051,6 +3358,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3092,6 +3404,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3133,6 +3450,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3174,6 +3496,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3215,6 +3542,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3256,6 +3588,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3297,6 +3634,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3336,6 +3678,11 @@
       <c r="K71" t="inlineStr">
         <is>
           <t>Growth Investment</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3379,6 +3726,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3418,6 +3770,11 @@
       <c r="K73" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3461,6 +3818,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3500,6 +3862,11 @@
       <c r="K75" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3543,6 +3910,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3584,6 +3956,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3625,6 +4002,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3666,6 +4048,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3705,6 +4092,11 @@
       <c r="K80" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -3748,6 +4140,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3789,6 +4186,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3830,6 +4232,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3871,6 +4278,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3912,6 +4324,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3953,6 +4370,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3994,6 +4416,11 @@
           <t>Balanced</t>
         </is>
       </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4035,6 +4462,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Liquidating Assets</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4076,6 +4508,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4117,6 +4554,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4158,6 +4600,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4197,6 +4644,11 @@
       <c r="K92" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
         </is>
       </c>
     </row>
@@ -4240,6 +4692,11 @@
           <t>Distress</t>
         </is>
       </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Growth Funded by Debt</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4281,6 +4738,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4322,6 +4784,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4363,6 +4830,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4404,6 +4876,11 @@
           <t>Growth Investment</t>
         </is>
       </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4445,6 +4922,11 @@
           <t>Deleveraging</t>
         </is>
       </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4486,6 +4968,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4527,6 +5014,11 @@
           <t>Asset Light</t>
         </is>
       </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4566,6 +5058,11 @@
       <c r="K101" t="inlineStr">
         <is>
           <t>Deleveraging</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>N/A</t>
         </is>
       </c>
     </row>

</xml_diff>